<commit_message>
Playbook budget: 2026 actuals from the operating budget
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PgxArtGdy89ocfVWD2QDDF
</commit_message>
<xml_diff>
--- a/site/assets/docs/fashion-lab-budget-template.xlsx
+++ b/site/assets/docs/fashion-lab-budget-template.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -477,7 +477,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Fashion Lab — Operating Budget Template (Sedona reference numbers, rounded)</t>
+          <t>Fashion Lab — Operating Budget Template (Sedona reference numbers, rounded; in-kind gifts not included)</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       <c r="D4" s="6" t="n"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Three sponsors in 2026</t>
+          <t>Five sponsors in 2026, $250 – $1,000 each</t>
         </is>
       </c>
     </row>
@@ -553,7 +553,7 @@
       <c r="D5" s="6" t="n"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>$1,500 per boutique; aim for three</t>
+          <t>$1,500 per boutique; one in 2026, aim for three</t>
         </is>
       </c>
     </row>
@@ -567,12 +567,12 @@
         <v>1800</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>1800</v>
+        <v>1600</v>
       </c>
       <c r="D6" s="6" t="n"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>$200 each; 12 is the target</t>
+          <t>$200 × 8 paid in 2026; 12 is the target</t>
         </is>
       </c>
     </row>
@@ -586,12 +586,12 @@
         <v>200</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>700</v>
+        <v>850</v>
       </c>
       <c r="D7" s="6" t="n"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>$50–$250 per ad</t>
+          <t>Five ads in 2026, $100 – $250 each</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
         <v>1580</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>1700</v>
+        <v>1600</v>
       </c>
       <c r="D8" s="6" t="n"/>
       <c r="E8" t="inlineStr">
@@ -629,7 +629,7 @@
       <c r="D9" s="6" t="n"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>$200 each</t>
+          <t>Four vendors in 2026; $200 a table</t>
         </is>
       </c>
     </row>
@@ -643,535 +643,608 @@
         <v>641</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>3555</v>
+        <v>5044</v>
       </c>
       <c r="D10" s="6" t="n"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Early bird $30, VIP $100</t>
+          <t>Mostly online; early bird $30, VIP $100. After $100 in refunds</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Raffle</t>
+          <t>Raffle &amp; bar</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
         <v>500</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>500</v>
+        <v>1856</v>
       </c>
       <c r="D11" s="6" t="n"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>10–12 high-end items</t>
+          <t>Raffle tickets plus drink sales on the night</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>City grant</t>
+          <t>Workshops</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>0</v>
+        <v>169</v>
       </c>
       <c r="D12" s="6" t="n"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Small community grant, year one</t>
+          <t>Pop-up workshop fees</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>City grant</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Small community grant; Sedona had one in 2025 only</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>TOTAL INCOME</t>
         </is>
       </c>
-      <c r="B13" s="7">
-        <f>SUM(B4:B12)</f>
-        <v/>
-      </c>
-      <c r="C13" s="7">
-        <f>SUM(C4:C12)</f>
-        <v/>
-      </c>
-      <c r="D13" s="7">
-        <f>SUM(D4:D12)</f>
-        <v/>
-      </c>
-      <c r="E13" s="2" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="B14" s="7">
+        <f>SUM(B4:B13)</f>
+        <v/>
+      </c>
+      <c r="C14" s="7">
+        <f>SUM(C4:C13)</f>
+        <v/>
+      </c>
+      <c r="D14" s="7">
+        <f>SUM(D4:D13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>EXPENSES · 48 Hour Create-a-Thon</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Studio / location</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Donated in Sedona (worth ~$2,000)</t>
-        </is>
-      </c>
+      <c r="B15" s="4" t="n"/>
+      <c r="C15" s="4" t="n"/>
+      <c r="D15" s="4" t="n"/>
+      <c r="E15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Location cleaning</t>
+          <t>Studio / location</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="D16" s="6" t="n"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Donated in Sedona (worth about $4,800)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Food for 48 hours</t>
+          <t>Location cleaning</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>441</v>
+        <v>200</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>490</v>
+        <v>250</v>
       </c>
       <c r="D17" s="6" t="n"/>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Get pizza donated</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Supplies</t>
+          <t>Food for 48 hours</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>157</v>
+        <v>441</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>281</v>
+        <v>589</v>
       </c>
       <c r="D18" s="6" t="n"/>
       <c r="E18" t="inlineStr">
         <is>
+          <t>Bulk snacks, two grocery runs and juice; get pizza donated</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Supplies (scissors, irons, thread)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>157</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>281</v>
+      </c>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" t="inlineStr">
+        <is>
           <t>More ironing boards than you think</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="B19" s="9">
-        <f>SUM(B15:B18)</f>
-        <v/>
-      </c>
-      <c r="C19" s="9">
-        <f>SUM(C15:C18)</f>
-        <v/>
-      </c>
-      <c r="D19" s="9">
-        <f>SUM(D15:D18)</f>
-        <v/>
-      </c>
-      <c r="E19" s="8" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="B20" s="7">
+        <f>SUM(B16:B19)</f>
+        <v/>
+      </c>
+      <c r="C20" s="7">
+        <f>SUM(C16:C19)</f>
+        <v/>
+      </c>
+      <c r="D20" s="7">
+        <f>SUM(D16:D19)</f>
+        <v/>
+      </c>
+      <c r="E20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>EXPENSES · Fashion Show</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="3" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Venue rental</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="n">
-        <v>1275</v>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>2500</v>
-      </c>
-      <c r="D21" s="6" t="n"/>
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Event insurance</t>
+          <t>Venue rental</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>263</v>
+        <v>1275</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>263</v>
+        <v>2500</v>
       </c>
       <c r="D22" s="6" t="n"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Hall + lobby + classroom, load-in to load-out</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Pipe and drape, runway</t>
+          <t>Event insurance</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>1564</v>
+        <v>263</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>1387</v>
+        <v>263</v>
       </c>
       <c r="D23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Pipe and drape, runway</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>0</v>
+        <v>1564</v>
       </c>
       <c r="C24" s="5" t="n">
-        <v>300</v>
+        <v>1387</v>
       </c>
       <c r="D24" s="6" t="n"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Rent more than you think</t>
+          <t>Local tent and event rental company</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>2040</v>
+        <v>375</v>
       </c>
       <c r="D25" s="6" t="n"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>A lighting tech for the night; rent more light than you think</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Photography</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>250</v>
+        <v>1500</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>250</v>
+        <v>1750</v>
       </c>
       <c r="D26" s="6" t="n"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Often partly donated</t>
+          <t>Show filming + reels</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Director / producer</t>
+          <t>Photography</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="C27" s="5" t="n">
         <v>500</v>
       </c>
       <c r="D27" s="6" t="n"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Two photographers, who also donated $1,000 of work</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>VIP reception</t>
+          <t>Director / producer</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>674</v>
+        <v>200</v>
       </c>
       <c r="C28" s="5" t="n">
-        <v>543</v>
+        <v>500</v>
       </c>
       <c r="D28" s="6" t="n"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>20 VIPs</t>
+          <t>Plus about $4,000 of donated time</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Trophy, raffle tickets, linens, signs</t>
+          <t>VIP reception &amp; bar (food, champagne, wine, beer, juice)</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>210</v>
+        <v>674</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>366</v>
+        <v>875</v>
       </c>
       <c r="D29" s="6" t="n"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>20 VIPs</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Jumbotron / screen</t>
+          <t>Trophy, raffle tickets, linens, signs, flowers, trash</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>0</v>
+        <v>210</v>
       </c>
       <c r="C30" s="5" t="n">
-        <v>500</v>
+        <v>978</v>
       </c>
       <c r="D30" s="6" t="n"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Small items add up</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Parking / shuttle</t>
+          <t>Jumbotron / screen</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>1400</v>
+        <v>0</v>
       </c>
       <c r="D31" s="6" t="n"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Only if the venue needs it</t>
+          <t>Optional; skipped in 2026</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>Parking / shuttle</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>2340</v>
+      </c>
+      <c r="D32" s="6" t="n"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Parking plus two shuttles. Only if your venue needs it</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Student helpers</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>230</v>
+      </c>
+      <c r="D33" s="6" t="n"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Local students helping backstage</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>Sales commissions</t>
         </is>
       </c>
-      <c r="B32" s="5" t="n">
+      <c r="B34" s="5" t="n">
         <v>965</v>
       </c>
-      <c r="C32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" s="6" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="C34" s="5" t="n">
+        <v>545</v>
+      </c>
+      <c r="D34" s="6" t="n"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>If someone sells sponsorships for you</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="B33" s="9">
-        <f>SUM(B21:B32)</f>
-        <v/>
-      </c>
-      <c r="C33" s="9">
-        <f>SUM(C21:C32)</f>
-        <v/>
-      </c>
-      <c r="D33" s="9">
-        <f>SUM(D21:D32)</f>
-        <v/>
-      </c>
-      <c r="E33" s="8" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+      <c r="B35" s="7">
+        <f>SUM(B22:B34)</f>
+        <v/>
+      </c>
+      <c r="C35" s="7">
+        <f>SUM(C22:C34)</f>
+        <v/>
+      </c>
+      <c r="D35" s="7">
+        <f>SUM(D22:D34)</f>
+        <v/>
+      </c>
+      <c r="E35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>EXPENSES · Award, publicity, online, pop-ups</t>
         </is>
       </c>
-      <c r="B34" s="4" t="n"/>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="4" t="n"/>
-      <c r="E34" s="3" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Cash scholarship</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C35" s="5" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D35" s="6" t="n"/>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>+ $4,000 courses donated by FABRIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Printing</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="n">
-        <v>786</v>
-      </c>
-      <c r="C36" s="5" t="n">
-        <v>1420</v>
-      </c>
-      <c r="D36" s="6" t="n"/>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>The printed program is the big one</t>
-        </is>
-      </c>
+      <c r="B36" s="4" t="n"/>
+      <c r="C36" s="4" t="n"/>
+      <c r="D36" s="4" t="n"/>
+      <c r="E36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Website hosting &amp; social scheduling</t>
+          <t>Cash scholarship &amp; prizes</t>
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>366</v>
+        <v>1000</v>
       </c>
       <c r="C37" s="5" t="n">
-        <v>296</v>
+        <v>1750</v>
       </c>
       <c r="D37" s="6" t="n"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>+ $8,000 in courses donated by FABRIC</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>Printing (cards, flyers, posters, tickets, program)</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>786</v>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>1420</v>
+      </c>
+      <c r="D38" s="6" t="n"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>The printed program is the big one</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Website hosting &amp; social scheduling</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>366</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>296</v>
+      </c>
+      <c r="D39" s="6" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>Pop-up events</t>
         </is>
       </c>
-      <c r="B38" s="5" t="n">
+      <c r="B40" s="5" t="n">
         <v>500</v>
       </c>
-      <c r="C38" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="6" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="B39" s="9">
-        <f>SUM(B35:B38)</f>
-        <v/>
-      </c>
-      <c r="C39" s="9">
-        <f>SUM(C35:C38)</f>
-        <v/>
-      </c>
-      <c r="D39" s="9">
-        <f>SUM(D35:D38)</f>
-        <v/>
-      </c>
-      <c r="E39" s="8" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL EXPENSES</t>
-        </is>
-      </c>
-      <c r="B40" s="7">
-        <f>B19+B33+B39</f>
-        <v/>
-      </c>
-      <c r="C40" s="7">
-        <f>C19+C33+C39</f>
-        <v/>
-      </c>
-      <c r="D40" s="7">
-        <f>D19+D33+D39</f>
-        <v/>
-      </c>
-      <c r="E40" s="2" t="n"/>
+      <c r="C40" s="5" t="n">
+        <v>400</v>
+      </c>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Workshop teachers</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="B41" s="7">
+        <f>SUM(B37:B40)</f>
+        <v/>
+      </c>
+      <c r="C41" s="7">
+        <f>SUM(C37:C40)</f>
+        <v/>
+      </c>
+      <c r="D41" s="7">
+        <f>SUM(D37:D40)</f>
+        <v/>
+      </c>
+      <c r="E41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL EXPENSES</t>
+        </is>
+      </c>
+      <c r="B42" s="7">
+        <f>B20+B35+B41</f>
+        <v/>
+      </c>
+      <c r="C42" s="7">
+        <f>C20+C35+C41</f>
+        <v/>
+      </c>
+      <c r="D42" s="7">
+        <f>D20+D35+D41</f>
+        <v/>
+      </c>
+      <c r="E42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
           <t>NET</t>
         </is>
       </c>
-      <c r="B41" s="7">
-        <f>B13-B40</f>
-        <v/>
-      </c>
-      <c r="C41" s="7">
-        <f>C13-C40</f>
-        <v/>
-      </c>
-      <c r="D41" s="7">
-        <f>D13-D40</f>
-        <v/>
-      </c>
-      <c r="E41" s="2" t="n"/>
+      <c r="B43" s="7">
+        <f>B14-B42</f>
+        <v/>
+      </c>
+      <c r="C43" s="7">
+        <f>C14-C42</f>
+        <v/>
+      </c>
+      <c r="D43" s="7">
+        <f>D14-D42</f>
+        <v/>
+      </c>
+      <c r="E43" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Playbook budget: 2026 actuals from the operating budget (#97)
Claude-Session: https://claude.ai/code/session_01PgxArtGdy89ocfVWD2QDDF

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/assets/docs/fashion-lab-budget-template.xlsx
+++ b/site/assets/docs/fashion-lab-budget-template.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -477,7 +477,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Fashion Lab — Operating Budget Template (Sedona reference numbers, rounded)</t>
+          <t>Fashion Lab — Operating Budget Template (Sedona reference numbers, rounded; in-kind gifts not included)</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       <c r="D4" s="6" t="n"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Three sponsors in 2026</t>
+          <t>Five sponsors in 2026, $250 – $1,000 each</t>
         </is>
       </c>
     </row>
@@ -553,7 +553,7 @@
       <c r="D5" s="6" t="n"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>$1,500 per boutique; aim for three</t>
+          <t>$1,500 per boutique; one in 2026, aim for three</t>
         </is>
       </c>
     </row>
@@ -567,12 +567,12 @@
         <v>1800</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>1800</v>
+        <v>1600</v>
       </c>
       <c r="D6" s="6" t="n"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>$200 each; 12 is the target</t>
+          <t>$200 × 8 paid in 2026; 12 is the target</t>
         </is>
       </c>
     </row>
@@ -586,12 +586,12 @@
         <v>200</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>700</v>
+        <v>850</v>
       </c>
       <c r="D7" s="6" t="n"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>$50–$250 per ad</t>
+          <t>Five ads in 2026, $100 – $250 each</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
         <v>1580</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>1700</v>
+        <v>1600</v>
       </c>
       <c r="D8" s="6" t="n"/>
       <c r="E8" t="inlineStr">
@@ -629,7 +629,7 @@
       <c r="D9" s="6" t="n"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>$200 each</t>
+          <t>Four vendors in 2026; $200 a table</t>
         </is>
       </c>
     </row>
@@ -643,535 +643,608 @@
         <v>641</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>3555</v>
+        <v>5044</v>
       </c>
       <c r="D10" s="6" t="n"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Early bird $30, VIP $100</t>
+          <t>Mostly online; early bird $30, VIP $100. After $100 in refunds</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Raffle</t>
+          <t>Raffle &amp; bar</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
         <v>500</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>500</v>
+        <v>1856</v>
       </c>
       <c r="D11" s="6" t="n"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>10–12 high-end items</t>
+          <t>Raffle tickets plus drink sales on the night</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>City grant</t>
+          <t>Workshops</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>0</v>
+        <v>169</v>
       </c>
       <c r="D12" s="6" t="n"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Small community grant, year one</t>
+          <t>Pop-up workshop fees</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>City grant</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Small community grant; Sedona had one in 2025 only</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>TOTAL INCOME</t>
         </is>
       </c>
-      <c r="B13" s="7">
-        <f>SUM(B4:B12)</f>
-        <v/>
-      </c>
-      <c r="C13" s="7">
-        <f>SUM(C4:C12)</f>
-        <v/>
-      </c>
-      <c r="D13" s="7">
-        <f>SUM(D4:D12)</f>
-        <v/>
-      </c>
-      <c r="E13" s="2" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="B14" s="7">
+        <f>SUM(B4:B13)</f>
+        <v/>
+      </c>
+      <c r="C14" s="7">
+        <f>SUM(C4:C13)</f>
+        <v/>
+      </c>
+      <c r="D14" s="7">
+        <f>SUM(D4:D13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>EXPENSES · 48 Hour Create-a-Thon</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Studio / location</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Donated in Sedona (worth ~$2,000)</t>
-        </is>
-      </c>
+      <c r="B15" s="4" t="n"/>
+      <c r="C15" s="4" t="n"/>
+      <c r="D15" s="4" t="n"/>
+      <c r="E15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Location cleaning</t>
+          <t>Studio / location</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="D16" s="6" t="n"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Donated in Sedona (worth about $4,800)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Food for 48 hours</t>
+          <t>Location cleaning</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>441</v>
+        <v>200</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>490</v>
+        <v>250</v>
       </c>
       <c r="D17" s="6" t="n"/>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Get pizza donated</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Supplies</t>
+          <t>Food for 48 hours</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>157</v>
+        <v>441</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>281</v>
+        <v>589</v>
       </c>
       <c r="D18" s="6" t="n"/>
       <c r="E18" t="inlineStr">
         <is>
+          <t>Bulk snacks, two grocery runs and juice; get pizza donated</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Supplies (scissors, irons, thread)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>157</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>281</v>
+      </c>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" t="inlineStr">
+        <is>
           <t>More ironing boards than you think</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="B19" s="9">
-        <f>SUM(B15:B18)</f>
-        <v/>
-      </c>
-      <c r="C19" s="9">
-        <f>SUM(C15:C18)</f>
-        <v/>
-      </c>
-      <c r="D19" s="9">
-        <f>SUM(D15:D18)</f>
-        <v/>
-      </c>
-      <c r="E19" s="8" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="B20" s="7">
+        <f>SUM(B16:B19)</f>
+        <v/>
+      </c>
+      <c r="C20" s="7">
+        <f>SUM(C16:C19)</f>
+        <v/>
+      </c>
+      <c r="D20" s="7">
+        <f>SUM(D16:D19)</f>
+        <v/>
+      </c>
+      <c r="E20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>EXPENSES · Fashion Show</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="3" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Venue rental</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="n">
-        <v>1275</v>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>2500</v>
-      </c>
-      <c r="D21" s="6" t="n"/>
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Event insurance</t>
+          <t>Venue rental</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>263</v>
+        <v>1275</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>263</v>
+        <v>2500</v>
       </c>
       <c r="D22" s="6" t="n"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Hall + lobby + classroom, load-in to load-out</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Pipe and drape, runway</t>
+          <t>Event insurance</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>1564</v>
+        <v>263</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>1387</v>
+        <v>263</v>
       </c>
       <c r="D23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Pipe and drape, runway</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>0</v>
+        <v>1564</v>
       </c>
       <c r="C24" s="5" t="n">
-        <v>300</v>
+        <v>1387</v>
       </c>
       <c r="D24" s="6" t="n"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Rent more than you think</t>
+          <t>Local tent and event rental company</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>2040</v>
+        <v>375</v>
       </c>
       <c r="D25" s="6" t="n"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>A lighting tech for the night; rent more light than you think</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Photography</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>250</v>
+        <v>1500</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>250</v>
+        <v>1750</v>
       </c>
       <c r="D26" s="6" t="n"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Often partly donated</t>
+          <t>Show filming + reels</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Director / producer</t>
+          <t>Photography</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="C27" s="5" t="n">
         <v>500</v>
       </c>
       <c r="D27" s="6" t="n"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Two photographers, who also donated $1,000 of work</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>VIP reception</t>
+          <t>Director / producer</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>674</v>
+        <v>200</v>
       </c>
       <c r="C28" s="5" t="n">
-        <v>543</v>
+        <v>500</v>
       </c>
       <c r="D28" s="6" t="n"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>20 VIPs</t>
+          <t>Plus about $4,000 of donated time</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Trophy, raffle tickets, linens, signs</t>
+          <t>VIP reception &amp; bar (food, champagne, wine, beer, juice)</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>210</v>
+        <v>674</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>366</v>
+        <v>875</v>
       </c>
       <c r="D29" s="6" t="n"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>20 VIPs</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Jumbotron / screen</t>
+          <t>Trophy, raffle tickets, linens, signs, flowers, trash</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>0</v>
+        <v>210</v>
       </c>
       <c r="C30" s="5" t="n">
-        <v>500</v>
+        <v>978</v>
       </c>
       <c r="D30" s="6" t="n"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Small items add up</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Parking / shuttle</t>
+          <t>Jumbotron / screen</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>1400</v>
+        <v>0</v>
       </c>
       <c r="D31" s="6" t="n"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Only if the venue needs it</t>
+          <t>Optional; skipped in 2026</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>Parking / shuttle</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>2340</v>
+      </c>
+      <c r="D32" s="6" t="n"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Parking plus two shuttles. Only if your venue needs it</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Student helpers</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>230</v>
+      </c>
+      <c r="D33" s="6" t="n"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Local students helping backstage</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>Sales commissions</t>
         </is>
       </c>
-      <c r="B32" s="5" t="n">
+      <c r="B34" s="5" t="n">
         <v>965</v>
       </c>
-      <c r="C32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" s="6" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="C34" s="5" t="n">
+        <v>545</v>
+      </c>
+      <c r="D34" s="6" t="n"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>If someone sells sponsorships for you</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="B33" s="9">
-        <f>SUM(B21:B32)</f>
-        <v/>
-      </c>
-      <c r="C33" s="9">
-        <f>SUM(C21:C32)</f>
-        <v/>
-      </c>
-      <c r="D33" s="9">
-        <f>SUM(D21:D32)</f>
-        <v/>
-      </c>
-      <c r="E33" s="8" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+      <c r="B35" s="7">
+        <f>SUM(B22:B34)</f>
+        <v/>
+      </c>
+      <c r="C35" s="7">
+        <f>SUM(C22:C34)</f>
+        <v/>
+      </c>
+      <c r="D35" s="7">
+        <f>SUM(D22:D34)</f>
+        <v/>
+      </c>
+      <c r="E35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>EXPENSES · Award, publicity, online, pop-ups</t>
         </is>
       </c>
-      <c r="B34" s="4" t="n"/>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="4" t="n"/>
-      <c r="E34" s="3" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Cash scholarship</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C35" s="5" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D35" s="6" t="n"/>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>+ $4,000 courses donated by FABRIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Printing</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="n">
-        <v>786</v>
-      </c>
-      <c r="C36" s="5" t="n">
-        <v>1420</v>
-      </c>
-      <c r="D36" s="6" t="n"/>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>The printed program is the big one</t>
-        </is>
-      </c>
+      <c r="B36" s="4" t="n"/>
+      <c r="C36" s="4" t="n"/>
+      <c r="D36" s="4" t="n"/>
+      <c r="E36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Website hosting &amp; social scheduling</t>
+          <t>Cash scholarship &amp; prizes</t>
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>366</v>
+        <v>1000</v>
       </c>
       <c r="C37" s="5" t="n">
-        <v>296</v>
+        <v>1750</v>
       </c>
       <c r="D37" s="6" t="n"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>+ $8,000 in courses donated by FABRIC</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>Printing (cards, flyers, posters, tickets, program)</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>786</v>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>1420</v>
+      </c>
+      <c r="D38" s="6" t="n"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>The printed program is the big one</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Website hosting &amp; social scheduling</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>366</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>296</v>
+      </c>
+      <c r="D39" s="6" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>Pop-up events</t>
         </is>
       </c>
-      <c r="B38" s="5" t="n">
+      <c r="B40" s="5" t="n">
         <v>500</v>
       </c>
-      <c r="C38" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="6" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="B39" s="9">
-        <f>SUM(B35:B38)</f>
-        <v/>
-      </c>
-      <c r="C39" s="9">
-        <f>SUM(C35:C38)</f>
-        <v/>
-      </c>
-      <c r="D39" s="9">
-        <f>SUM(D35:D38)</f>
-        <v/>
-      </c>
-      <c r="E39" s="8" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL EXPENSES</t>
-        </is>
-      </c>
-      <c r="B40" s="7">
-        <f>B19+B33+B39</f>
-        <v/>
-      </c>
-      <c r="C40" s="7">
-        <f>C19+C33+C39</f>
-        <v/>
-      </c>
-      <c r="D40" s="7">
-        <f>D19+D33+D39</f>
-        <v/>
-      </c>
-      <c r="E40" s="2" t="n"/>
+      <c r="C40" s="5" t="n">
+        <v>400</v>
+      </c>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Workshop teachers</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="B41" s="7">
+        <f>SUM(B37:B40)</f>
+        <v/>
+      </c>
+      <c r="C41" s="7">
+        <f>SUM(C37:C40)</f>
+        <v/>
+      </c>
+      <c r="D41" s="7">
+        <f>SUM(D37:D40)</f>
+        <v/>
+      </c>
+      <c r="E41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL EXPENSES</t>
+        </is>
+      </c>
+      <c r="B42" s="7">
+        <f>B20+B35+B41</f>
+        <v/>
+      </c>
+      <c r="C42" s="7">
+        <f>C20+C35+C41</f>
+        <v/>
+      </c>
+      <c r="D42" s="7">
+        <f>D20+D35+D41</f>
+        <v/>
+      </c>
+      <c r="E42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
           <t>NET</t>
         </is>
       </c>
-      <c r="B41" s="7">
-        <f>B13-B40</f>
-        <v/>
-      </c>
-      <c r="C41" s="7">
-        <f>C13-C40</f>
-        <v/>
-      </c>
-      <c r="D41" s="7">
-        <f>D13-D40</f>
-        <v/>
-      </c>
-      <c r="E41" s="2" t="n"/>
+      <c r="B43" s="7">
+        <f>B14-B42</f>
+        <v/>
+      </c>
+      <c r="C43" s="7">
+        <f>C14-C42</f>
+        <v/>
+      </c>
+      <c r="D43" s="7">
+        <f>D14-D42</f>
+        <v/>
+      </c>
+      <c r="E43" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Playbook budget: VIP Models line name; download gets the planner tab
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PgxArtGdy89ocfVWD2QDDF
</commit_message>
<xml_diff>
--- a/site/assets/docs/fashion-lab-budget-template.xlsx
+++ b/site/assets/docs/fashion-lab-budget-template.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget template" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sedona budget" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan by size" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -78,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -99,6 +100,12 @@
     <xf numFmtId="164" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -464,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -560,7 +567,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sensational Sedonans (program ads)</t>
+          <t>VIP Models – Sensational Sedonans + Ad in the Program</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
@@ -1245,6 +1252,74 @@
         <v/>
       </c>
       <c r="E43" s="2" t="n"/>
+    </row>
+    <row r="44"/>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>YEAR 1 (2024), cash vs. donated</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Cash spent</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="n">
+        <v>2770</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Food, supplies, printing, VIP party</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Donated</t>
+        </is>
+      </c>
+      <c r="B47" s="11" t="n">
+        <v>6100</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Venue, sound / DJ, production help</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Traded</t>
+        </is>
+      </c>
+      <c r="B48" s="11" t="n">
+        <v>997</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Venue hours swapped for services</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Value of the first show</t>
+        </is>
+      </c>
+      <c r="B49" s="11" t="n">
+        <v>10155</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Before discounts and donations</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1252,6 +1327,502 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Plan by size: change the yellow cells, the rest works itself out</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr"/>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>INPUTS</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="n"/>
+      <c r="C4" s="12" t="n"/>
+      <c r="D4" s="12" t="n"/>
+      <c r="E4" s="12" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Designers</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="D5" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Create-a-Thon participants</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Designer registration</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="D6" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Per designer</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Regular tickets sold</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>About one per designer to start</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Regular ticket price</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>33</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>33</v>
+      </c>
+      <c r="D8" s="14" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>VIP tickets sold</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="D9" s="13" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>VIP ticket price</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Includes the pre-show reception</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Food per designer, whole weekend</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>65</v>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="D11" s="14" t="n">
+        <v>130</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Dinner, lunch, breakfast, snacks</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Supplies per designer</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="D12" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Thread, notions, irons, scissors</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="n">
+        <v>500</v>
+      </c>
+      <c r="C13" s="14" t="n">
+        <v>500</v>
+      </c>
+      <c r="D13" s="14" t="n">
+        <v>500</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Often donated</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Other fixed costs</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Cake, signs, small items</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>INCOME</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="12" t="n"/>
+      <c r="D15" s="12" t="n"/>
+      <c r="E15" s="12" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Registrations</t>
+        </is>
+      </c>
+      <c r="B16" s="11">
+        <f>B5*B6</f>
+        <v/>
+      </c>
+      <c r="C16" s="11">
+        <f>C5*C6</f>
+        <v/>
+      </c>
+      <c r="D16" s="11">
+        <f>D5*D6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Tickets</t>
+        </is>
+      </c>
+      <c r="B17" s="11">
+        <f>B7*B8+B9*B10</f>
+        <v/>
+      </c>
+      <c r="C17" s="11">
+        <f>C7*C8+C9*C10</f>
+        <v/>
+      </c>
+      <c r="D17" s="11">
+        <f>D7*D8+D9*D10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Total income</t>
+        </is>
+      </c>
+      <c r="B18" s="15">
+        <f>B16+B17</f>
+        <v/>
+      </c>
+      <c r="C18" s="15">
+        <f>C16+C17</f>
+        <v/>
+      </c>
+      <c r="D18" s="15">
+        <f>D16+D17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>COSTS</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="n"/>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="12" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="B20" s="11">
+        <f>B5*B11</f>
+        <v/>
+      </c>
+      <c r="C20" s="11">
+        <f>C5*C11</f>
+        <v/>
+      </c>
+      <c r="D20" s="11">
+        <f>D5*D11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="B21" s="11">
+        <f>B5*B12</f>
+        <v/>
+      </c>
+      <c r="C21" s="11">
+        <f>C5*C12</f>
+        <v/>
+      </c>
+      <c r="D21" s="11">
+        <f>D5*D12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="B22" s="11">
+        <f>B13</f>
+        <v/>
+      </c>
+      <c r="C22" s="11">
+        <f>C13</f>
+        <v/>
+      </c>
+      <c r="D22" s="11">
+        <f>D13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B23" s="11">
+        <f>B14</f>
+        <v/>
+      </c>
+      <c r="C23" s="11">
+        <f>C14</f>
+        <v/>
+      </c>
+      <c r="D23" s="11">
+        <f>D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Total costs</t>
+        </is>
+      </c>
+      <c r="B24" s="15">
+        <f>SUM(B20:B23)</f>
+        <v/>
+      </c>
+      <c r="C24" s="15">
+        <f>SUM(C20:C23)</f>
+        <v/>
+      </c>
+      <c r="D24" s="15">
+        <f>SUM(D20:D23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>RESULT</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="n"/>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="12" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Cost per designer</t>
+        </is>
+      </c>
+      <c r="B26" s="15">
+        <f>B24/B5</f>
+        <v/>
+      </c>
+      <c r="C26" s="15">
+        <f>C24/C5</f>
+        <v/>
+      </c>
+      <c r="D26" s="15">
+        <f>D24/D5</f>
+        <v/>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>What each designer costs to host</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Sponsorship needed</t>
+        </is>
+      </c>
+      <c r="B27" s="15">
+        <f>MAX(0,B24-B18)</f>
+        <v/>
+      </c>
+      <c r="C27" s="15">
+        <f>MAX(0,C24-C18)</f>
+        <v/>
+      </c>
+      <c r="D27" s="15">
+        <f>MAX(0,D24-D18)</f>
+        <v/>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>The gap sponsors, ads and vendors fill</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1406,7 +1977,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Playbook budget: Title Case line labels
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PgxArtGdy89ocfVWD2QDDF
</commit_message>
<xml_diff>
--- a/site/assets/docs/fashion-lab-budget-template.xlsx
+++ b/site/assets/docs/fashion-lab-budget-template.xlsx
@@ -529,7 +529,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Event sponsors &amp; underwriters</t>
+          <t>Event Sponsors &amp; Underwriters</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
@@ -548,7 +548,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Boutique sponsors</t>
+          <t>Boutique Sponsors</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
@@ -586,7 +586,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Program ads</t>
+          <t>Program Ads</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
@@ -605,7 +605,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Designer registrations</t>
+          <t>Designer Registrations</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
@@ -624,7 +624,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Vendor tables</t>
+          <t>Vendor Tables</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
@@ -662,7 +662,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Raffle &amp; bar</t>
+          <t>Raffle &amp; Bar</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
@@ -700,7 +700,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>City grant</t>
+          <t>City Grant</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
@@ -750,7 +750,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Studio / location</t>
+          <t>Studio / Location</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
@@ -769,7 +769,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Location cleaning</t>
+          <t>Location Cleaning</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
@@ -783,7 +783,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Food for 48 hours</t>
+          <t>Food for 48 Hours</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
@@ -802,7 +802,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Supplies (scissors, irons, thread)</t>
+          <t>Supplies (Scissors, Irons, Thread)</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
@@ -852,7 +852,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Venue rental</t>
+          <t>Venue Rental</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
@@ -871,7 +871,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Event insurance</t>
+          <t>Event Insurance</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
@@ -885,7 +885,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Pipe and drape, runway</t>
+          <t>Pipe and Drape, Runway</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
@@ -961,7 +961,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Director / producer</t>
+          <t>Director / Producer</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
@@ -980,7 +980,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>VIP reception &amp; bar (food, champagne, wine, beer, juice)</t>
+          <t>VIP Reception &amp; Bar (Food, Champagne, Wine, Beer, Juice)</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
@@ -999,7 +999,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Trophy, raffle tickets, linens, signs, flowers, trash</t>
+          <t>Trophy, Raffle Tickets, Linens, Signs, Flowers, Trash</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
@@ -1018,7 +1018,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jumbotron / screen</t>
+          <t>Jumbotron / Screen</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
@@ -1037,7 +1037,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Parking / shuttle</t>
+          <t>Parking / Shuttle</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
@@ -1056,7 +1056,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Student helpers</t>
+          <t>Student Helpers</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
@@ -1075,7 +1075,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Sales commissions</t>
+          <t>Sales Commissions</t>
         </is>
       </c>
       <c r="B34" s="5" t="n">
@@ -1114,7 +1114,7 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>EXPENSES · Award, publicity, online, pop-ups</t>
+          <t>EXPENSES · Award, Publicity, Online, Pop-ups</t>
         </is>
       </c>
       <c r="B36" s="4" t="n"/>
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cash scholarship &amp; prizes</t>
+          <t>Cash Scholarship &amp; Prizes</t>
         </is>
       </c>
       <c r="B37" s="5" t="n">
@@ -1144,7 +1144,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Printing (cards, flyers, posters, tickets, program)</t>
+          <t>Printing (Cards, Flyers, Posters, Tickets, Program)</t>
         </is>
       </c>
       <c r="B38" s="5" t="n">
@@ -1163,7 +1163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Website hosting &amp; social scheduling</t>
+          <t>Website Hosting &amp; Social Scheduling</t>
         </is>
       </c>
       <c r="B39" s="5" t="n">
@@ -1177,7 +1177,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Pop-up events</t>
+          <t>Pop-Up Events</t>
         </is>
       </c>
       <c r="B40" s="5" t="n">
@@ -1257,14 +1257,14 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>YEAR 1 (2024), cash vs. donated</t>
+          <t>YEAR 1 (2024), Cash vs. Donated</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Cash spent</t>
+          <t>Cash Spent</t>
         </is>
       </c>
       <c r="B46" s="11" t="n">
@@ -1309,7 +1309,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Value of the first show</t>
+          <t>Value of the First Show</t>
         </is>
       </c>
       <c r="B49" s="11" t="n">
@@ -1408,7 +1408,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Designer registration</t>
+          <t>Designer Registration</t>
         </is>
       </c>
       <c r="B6" s="14" t="n">
@@ -1429,7 +1429,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Regular tickets sold</t>
+          <t>Regular Tickets Sold</t>
         </is>
       </c>
       <c r="B7" s="13" t="n">
@@ -1450,7 +1450,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Regular ticket price</t>
+          <t>Regular Ticket Price</t>
         </is>
       </c>
       <c r="B8" s="14" t="n">
@@ -1466,7 +1466,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>VIP tickets sold</t>
+          <t>VIP Tickets Sold</t>
         </is>
       </c>
       <c r="B9" s="13" t="n">
@@ -1482,7 +1482,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>VIP ticket price</t>
+          <t>VIP Ticket Price</t>
         </is>
       </c>
       <c r="B10" s="14" t="n">
@@ -1503,7 +1503,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Food per designer, whole weekend</t>
+          <t>Food per Designer, Whole Weekend</t>
         </is>
       </c>
       <c r="B11" s="14" t="n">
@@ -1524,7 +1524,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Supplies per designer</t>
+          <t>Supplies per Designer</t>
         </is>
       </c>
       <c r="B12" s="14" t="n">
@@ -1566,7 +1566,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Other fixed costs</t>
+          <t>Other Fixed Costs</t>
         </is>
       </c>
       <c r="B14" s="14" t="n">
@@ -1636,7 +1636,7 @@
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>Total income</t>
+          <t>Total Income</t>
         </is>
       </c>
       <c r="B18" s="15">
@@ -1742,7 +1742,7 @@
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>Total costs</t>
+          <t>Total Costs</t>
         </is>
       </c>
       <c r="B24" s="15">
@@ -1772,7 +1772,7 @@
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>Cost per designer</t>
+          <t>Cost per Designer</t>
         </is>
       </c>
       <c r="B26" s="15">
@@ -1796,7 +1796,7 @@
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>Sponsorship needed</t>
+          <t>Sponsorship Needed</t>
         </is>
       </c>
       <c r="B27" s="15">

</xml_diff>

<commit_message>
Playbook budget: VIP Models line, Title Case labels, planner in the download (#100)
* Playbook budget: VIP Models line name; download gets the planner tab

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PgxArtGdy89ocfVWD2QDDF

* Playbook budget: Title Case line labels

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PgxArtGdy89ocfVWD2QDDF

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/assets/docs/fashion-lab-budget-template.xlsx
+++ b/site/assets/docs/fashion-lab-budget-template.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget template" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sedona budget" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan by size" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -78,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -99,6 +100,12 @@
     <xf numFmtId="164" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -464,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -522,7 +529,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Event sponsors &amp; underwriters</t>
+          <t>Event Sponsors &amp; Underwriters</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
@@ -541,7 +548,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Boutique sponsors</t>
+          <t>Boutique Sponsors</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
@@ -560,7 +567,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sensational Sedonans (program ads)</t>
+          <t>VIP Models – Sensational Sedonans + Ad in the Program</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
@@ -579,7 +586,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Program ads</t>
+          <t>Program Ads</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
@@ -598,7 +605,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Designer registrations</t>
+          <t>Designer Registrations</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
@@ -617,7 +624,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Vendor tables</t>
+          <t>Vendor Tables</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
@@ -655,7 +662,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Raffle &amp; bar</t>
+          <t>Raffle &amp; Bar</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
@@ -693,7 +700,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>City grant</t>
+          <t>City Grant</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
@@ -743,7 +750,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Studio / location</t>
+          <t>Studio / Location</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
@@ -762,7 +769,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Location cleaning</t>
+          <t>Location Cleaning</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
@@ -776,7 +783,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Food for 48 hours</t>
+          <t>Food for 48 Hours</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
@@ -795,7 +802,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Supplies (scissors, irons, thread)</t>
+          <t>Supplies (Scissors, Irons, Thread)</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
@@ -845,7 +852,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Venue rental</t>
+          <t>Venue Rental</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
@@ -864,7 +871,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Event insurance</t>
+          <t>Event Insurance</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
@@ -878,7 +885,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Pipe and drape, runway</t>
+          <t>Pipe and Drape, Runway</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
@@ -954,7 +961,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Director / producer</t>
+          <t>Director / Producer</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
@@ -973,7 +980,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>VIP reception &amp; bar (food, champagne, wine, beer, juice)</t>
+          <t>VIP Reception &amp; Bar (Food, Champagne, Wine, Beer, Juice)</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
@@ -992,7 +999,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Trophy, raffle tickets, linens, signs, flowers, trash</t>
+          <t>Trophy, Raffle Tickets, Linens, Signs, Flowers, Trash</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
@@ -1011,7 +1018,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jumbotron / screen</t>
+          <t>Jumbotron / Screen</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
@@ -1030,7 +1037,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Parking / shuttle</t>
+          <t>Parking / Shuttle</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
@@ -1049,7 +1056,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Student helpers</t>
+          <t>Student Helpers</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
@@ -1068,7 +1075,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Sales commissions</t>
+          <t>Sales Commissions</t>
         </is>
       </c>
       <c r="B34" s="5" t="n">
@@ -1107,7 +1114,7 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>EXPENSES · Award, publicity, online, pop-ups</t>
+          <t>EXPENSES · Award, Publicity, Online, Pop-ups</t>
         </is>
       </c>
       <c r="B36" s="4" t="n"/>
@@ -1118,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cash scholarship &amp; prizes</t>
+          <t>Cash Scholarship &amp; Prizes</t>
         </is>
       </c>
       <c r="B37" s="5" t="n">
@@ -1137,7 +1144,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Printing (cards, flyers, posters, tickets, program)</t>
+          <t>Printing (Cards, Flyers, Posters, Tickets, Program)</t>
         </is>
       </c>
       <c r="B38" s="5" t="n">
@@ -1156,7 +1163,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Website hosting &amp; social scheduling</t>
+          <t>Website Hosting &amp; Social Scheduling</t>
         </is>
       </c>
       <c r="B39" s="5" t="n">
@@ -1170,7 +1177,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Pop-up events</t>
+          <t>Pop-Up Events</t>
         </is>
       </c>
       <c r="B40" s="5" t="n">
@@ -1245,6 +1252,74 @@
         <v/>
       </c>
       <c r="E43" s="2" t="n"/>
+    </row>
+    <row r="44"/>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>YEAR 1 (2024), Cash vs. Donated</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Cash Spent</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="n">
+        <v>2770</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Food, supplies, printing, VIP party</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Donated</t>
+        </is>
+      </c>
+      <c r="B47" s="11" t="n">
+        <v>6100</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Venue, sound / DJ, production help</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Traded</t>
+        </is>
+      </c>
+      <c r="B48" s="11" t="n">
+        <v>997</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Venue hours swapped for services</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Value of the First Show</t>
+        </is>
+      </c>
+      <c r="B49" s="11" t="n">
+        <v>10155</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Before discounts and donations</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1252,6 +1327,502 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Plan by size: change the yellow cells, the rest works itself out</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr"/>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>INPUTS</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="n"/>
+      <c r="C4" s="12" t="n"/>
+      <c r="D4" s="12" t="n"/>
+      <c r="E4" s="12" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Designers</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="D5" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Create-a-Thon participants</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Designer Registration</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="D6" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Per designer</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Regular Tickets Sold</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>About one per designer to start</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Regular Ticket Price</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>33</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>33</v>
+      </c>
+      <c r="D8" s="14" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>VIP Tickets Sold</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="D9" s="13" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>VIP Ticket Price</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Includes the pre-show reception</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Food per Designer, Whole Weekend</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>65</v>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="D11" s="14" t="n">
+        <v>130</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Dinner, lunch, breakfast, snacks</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Supplies per Designer</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="D12" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Thread, notions, irons, scissors</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="n">
+        <v>500</v>
+      </c>
+      <c r="C13" s="14" t="n">
+        <v>500</v>
+      </c>
+      <c r="D13" s="14" t="n">
+        <v>500</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Often donated</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Other Fixed Costs</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Cake, signs, small items</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>INCOME</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="12" t="n"/>
+      <c r="D15" s="12" t="n"/>
+      <c r="E15" s="12" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Registrations</t>
+        </is>
+      </c>
+      <c r="B16" s="11">
+        <f>B5*B6</f>
+        <v/>
+      </c>
+      <c r="C16" s="11">
+        <f>C5*C6</f>
+        <v/>
+      </c>
+      <c r="D16" s="11">
+        <f>D5*D6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Tickets</t>
+        </is>
+      </c>
+      <c r="B17" s="11">
+        <f>B7*B8+B9*B10</f>
+        <v/>
+      </c>
+      <c r="C17" s="11">
+        <f>C7*C8+C9*C10</f>
+        <v/>
+      </c>
+      <c r="D17" s="11">
+        <f>D7*D8+D9*D10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Total Income</t>
+        </is>
+      </c>
+      <c r="B18" s="15">
+        <f>B16+B17</f>
+        <v/>
+      </c>
+      <c r="C18" s="15">
+        <f>C16+C17</f>
+        <v/>
+      </c>
+      <c r="D18" s="15">
+        <f>D16+D17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>COSTS</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="n"/>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="12" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="B20" s="11">
+        <f>B5*B11</f>
+        <v/>
+      </c>
+      <c r="C20" s="11">
+        <f>C5*C11</f>
+        <v/>
+      </c>
+      <c r="D20" s="11">
+        <f>D5*D11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="B21" s="11">
+        <f>B5*B12</f>
+        <v/>
+      </c>
+      <c r="C21" s="11">
+        <f>C5*C12</f>
+        <v/>
+      </c>
+      <c r="D21" s="11">
+        <f>D5*D12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="B22" s="11">
+        <f>B13</f>
+        <v/>
+      </c>
+      <c r="C22" s="11">
+        <f>C13</f>
+        <v/>
+      </c>
+      <c r="D22" s="11">
+        <f>D13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B23" s="11">
+        <f>B14</f>
+        <v/>
+      </c>
+      <c r="C23" s="11">
+        <f>C14</f>
+        <v/>
+      </c>
+      <c r="D23" s="11">
+        <f>D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Total Costs</t>
+        </is>
+      </c>
+      <c r="B24" s="15">
+        <f>SUM(B20:B23)</f>
+        <v/>
+      </c>
+      <c r="C24" s="15">
+        <f>SUM(C20:C23)</f>
+        <v/>
+      </c>
+      <c r="D24" s="15">
+        <f>SUM(D20:D23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>RESULT</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="n"/>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="12" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Cost per Designer</t>
+        </is>
+      </c>
+      <c r="B26" s="15">
+        <f>B24/B5</f>
+        <v/>
+      </c>
+      <c r="C26" s="15">
+        <f>C24/C5</f>
+        <v/>
+      </c>
+      <c r="D26" s="15">
+        <f>D24/D5</f>
+        <v/>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>What each designer costs to host</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Sponsorship Needed</t>
+        </is>
+      </c>
+      <c r="B27" s="15">
+        <f>MAX(0,B24-B18)</f>
+        <v/>
+      </c>
+      <c r="C27" s="15">
+        <f>MAX(0,C24-C18)</f>
+        <v/>
+      </c>
+      <c r="D27" s="15">
+        <f>MAX(0,D24-D18)</f>
+        <v/>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>The gap sponsors, ads and vendors fill</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1406,7 +1977,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Playbook budget: how-many × price calculators, raffle + bar line
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PgxArtGdy89ocfVWD2QDDF
</commit_message>
<xml_diff>
--- a/site/assets/docs/fashion-lab-budget-template.xlsx
+++ b/site/assets/docs/fashion-lab-budget-template.xlsx
@@ -79,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -106,6 +106,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -471,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -479,6 +482,8 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -514,6 +519,16 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Your #</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Price each</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -557,11 +572,18 @@
       <c r="C5" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="D5" s="6" t="n"/>
+      <c r="D5" s="6">
+        <f>IF(F5="","",F5*G5)</f>
+        <v/>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>$1,500 per boutique; one in 2026, aim for three</t>
-        </is>
+          <t>One in 2026; aim for three. Type how many in column F</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="11" t="n">
+        <v>1500</v>
       </c>
     </row>
     <row r="6">
@@ -576,11 +598,18 @@
       <c r="C6" s="5" t="n">
         <v>1600</v>
       </c>
-      <c r="D6" s="6" t="n"/>
+      <c r="D6" s="6">
+        <f>IF(F6="","",F6*G6)</f>
+        <v/>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>$200 × 8 paid in 2026; 12 is the target</t>
-        </is>
+          <t>Eight paid in 2026; 12 is the target. Type how many in column F</t>
+        </is>
+      </c>
+      <c r="F6" s="16" t="n"/>
+      <c r="G6" s="11" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="7">
@@ -614,11 +643,18 @@
       <c r="C8" s="5" t="n">
         <v>1600</v>
       </c>
-      <c r="D8" s="6" t="n"/>
+      <c r="D8" s="6">
+        <f>IF(F8="","",F8*G8)</f>
+        <v/>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>$100 each</t>
-        </is>
+          <t>Sixteen paid in 2026. Type how many in column F</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="n"/>
+      <c r="G8" s="11" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="9">
@@ -633,11 +669,18 @@
       <c r="C9" s="5" t="n">
         <v>1250</v>
       </c>
-      <c r="D9" s="6" t="n"/>
+      <c r="D9" s="6">
+        <f>IF(F9="","",F9*G9)</f>
+        <v/>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Four vendors in 2026; $200 a table</t>
-        </is>
+          <t>Four vendors in 2026, some took bigger spots. Type how many in column F</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="n"/>
+      <c r="G9" s="11" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="10">
@@ -662,7 +705,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Raffle &amp; Bar</t>
+          <t>Raffle + Bar / Juice Bar / Nibbles</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
@@ -674,7 +717,7 @@
       <c r="D11" s="6" t="n"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Raffle tickets plus drink sales on the night</t>
+          <t>Sold together; the bar is roughly a third to a half of it. Raffle: 1 for $5, 3 for $10, 9 for $20</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1392,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="10" t="inlineStr"/>
       <c r="B3" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Playbook budget: how-many × price calculators, raffle + bar line (#101)
Claude-Session: https://claude.ai/code/session_01PgxArtGdy89ocfVWD2QDDF

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/assets/docs/fashion-lab-budget-template.xlsx
+++ b/site/assets/docs/fashion-lab-budget-template.xlsx
@@ -79,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -106,6 +106,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -471,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -479,6 +482,8 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -514,6 +519,16 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Your #</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Price each</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -557,11 +572,18 @@
       <c r="C5" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="D5" s="6" t="n"/>
+      <c r="D5" s="6">
+        <f>IF(F5="","",F5*G5)</f>
+        <v/>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>$1,500 per boutique; one in 2026, aim for three</t>
-        </is>
+          <t>One in 2026; aim for three. Type how many in column F</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="11" t="n">
+        <v>1500</v>
       </c>
     </row>
     <row r="6">
@@ -576,11 +598,18 @@
       <c r="C6" s="5" t="n">
         <v>1600</v>
       </c>
-      <c r="D6" s="6" t="n"/>
+      <c r="D6" s="6">
+        <f>IF(F6="","",F6*G6)</f>
+        <v/>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>$200 × 8 paid in 2026; 12 is the target</t>
-        </is>
+          <t>Eight paid in 2026; 12 is the target. Type how many in column F</t>
+        </is>
+      </c>
+      <c r="F6" s="16" t="n"/>
+      <c r="G6" s="11" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="7">
@@ -614,11 +643,18 @@
       <c r="C8" s="5" t="n">
         <v>1600</v>
       </c>
-      <c r="D8" s="6" t="n"/>
+      <c r="D8" s="6">
+        <f>IF(F8="","",F8*G8)</f>
+        <v/>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>$100 each</t>
-        </is>
+          <t>Sixteen paid in 2026. Type how many in column F</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="n"/>
+      <c r="G8" s="11" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="9">
@@ -633,11 +669,18 @@
       <c r="C9" s="5" t="n">
         <v>1250</v>
       </c>
-      <c r="D9" s="6" t="n"/>
+      <c r="D9" s="6">
+        <f>IF(F9="","",F9*G9)</f>
+        <v/>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Four vendors in 2026; $200 a table</t>
-        </is>
+          <t>Four vendors in 2026, some took bigger spots. Type how many in column F</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="n"/>
+      <c r="G9" s="11" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="10">
@@ -662,7 +705,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Raffle &amp; Bar</t>
+          <t>Raffle + Bar / Juice Bar / Nibbles</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
@@ -674,7 +717,7 @@
       <c r="D11" s="6" t="n"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Raffle tickets plus drink sales on the night</t>
+          <t>Sold together; the bar is roughly a third to a half of it. Raffle: 1 for $5, 3 for $10, 9 for $20</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1392,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="10" t="inlineStr"/>
       <c r="B3" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Playbook budget: summary top and bottom, cost per designer, donations, prior surplus, saved in browser, CSV download
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PgxArtGdy89ocfVWD2QDDF
</commit_message>
<xml_diff>
--- a/site/assets/docs/fashion-lab-budget-template.xlsx
+++ b/site/assets/docs/fashion-lab-budget-template.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1296,69 +1296,264 @@
       </c>
       <c r="E43" s="2" t="n"/>
     </row>
-    <row r="44"/>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>COST PER DESIGNER</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="n"/>
+      <c r="C44" s="7">
+        <f>C42/16</f>
+        <v/>
+      </c>
+      <c r="D44" s="7">
+        <f>IF(OR(F8="",F8=0),"",D42/F8)</f>
+        <v/>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Expenses ÷ designers (Sedona 2026 had 16 paying designers)</t>
+        </is>
+      </c>
+    </row>
     <row r="45">
-      <c r="A45" s="10" t="inlineStr">
-        <is>
-          <t>YEAR 1 (2024), Cash vs. Donated</t>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Surplus From Prior Year</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n"/>
+      <c r="C45" s="5" t="n">
+        <v>5083</v>
+      </c>
+      <c r="D45" s="6" t="n"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>What was left in the bank from last year</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Cash Spent</t>
-        </is>
-      </c>
-      <c r="B46" s="11" t="n">
-        <v>2770</v>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Food, supplies, printing, VIP party</t>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>IN THE BANK AFTER</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="n"/>
+      <c r="C46" s="7">
+        <f>C45+C43</f>
+        <v/>
+      </c>
+      <c r="D46" s="7">
+        <f>D45+D43</f>
+        <v/>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Prior surplus + net. Sedona carried $4,723 into 2027</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Donated</t>
-        </is>
-      </c>
-      <c r="B47" s="11" t="n">
-        <v>6100</v>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Venue, sound / DJ, production help</t>
-        </is>
-      </c>
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>DONATED (IN-KIND) · not in the cash totals</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="n"/>
+      <c r="C47" s="4" t="n"/>
+      <c r="D47" s="4" t="n"/>
+      <c r="E47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Traded</t>
-        </is>
-      </c>
-      <c r="B48" s="11" t="n">
-        <v>997</v>
-      </c>
+          <t>Create-a-Thon Studio</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n"/>
+      <c r="C48" s="5" t="n">
+        <v>4800</v>
+      </c>
+      <c r="D48" s="6" t="n"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Venue hours swapped for services</t>
+          <t>Weekend studio space</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>Scholarship Courses &amp; Mentorship</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n"/>
+      <c r="C49" s="5" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D49" s="6" t="n"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Donated by the FABRIC Incubator</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Raffle Prizes</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n"/>
+      <c r="C50" s="5" t="n">
+        <v>6941</v>
+      </c>
+      <c r="D50" s="6" t="n"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>High-end items from local businesses</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Director / Producer Time</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n"/>
+      <c r="C51" s="5" t="n">
+        <v>4000</v>
+      </c>
+      <c r="D51" s="6" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n"/>
+      <c r="C52" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D52" s="6" t="n"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Two photographers</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Stage Manager</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n"/>
+      <c r="C53" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="D53" s="6" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n"/>
+      <c r="C54" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="D54" s="6" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>SAVED BY DONATIONS</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="n"/>
+      <c r="C55" s="7">
+        <f>SUM(C48:C54)</f>
+        <v/>
+      </c>
+      <c r="D55" s="7">
+        <f>SUM(D48:D54)</f>
+        <v/>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>What you didn't have to pay for</t>
+        </is>
+      </c>
+    </row>
+    <row r="56"/>
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>YEAR 1 (2024), Cash vs. Donated</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Cash Spent</t>
+        </is>
+      </c>
+      <c r="B58" s="11" t="n">
+        <v>2770</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Food, supplies, printing, VIP party</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Donated</t>
+        </is>
+      </c>
+      <c r="B59" s="11" t="n">
+        <v>6100</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Venue, sound / DJ, production help</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Traded</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="n">
+        <v>997</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Venue hours swapped for services</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>Value of the First Show</t>
         </is>
       </c>
-      <c r="B49" s="11" t="n">
+      <c r="B61" s="11" t="n">
         <v>10155</v>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>Before discounts and donations</t>
         </is>

</xml_diff>

<commit_message>
Playbook budget: summary top and bottom, cost per designer, donations, prior surplus, saved in browser, CSV download (#103)
Claude-Session: https://claude.ai/code/session_01PgxArtGdy89ocfVWD2QDDF

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/assets/docs/fashion-lab-budget-template.xlsx
+++ b/site/assets/docs/fashion-lab-budget-template.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1296,69 +1296,264 @@
       </c>
       <c r="E43" s="2" t="n"/>
     </row>
-    <row r="44"/>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>COST PER DESIGNER</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="n"/>
+      <c r="C44" s="7">
+        <f>C42/16</f>
+        <v/>
+      </c>
+      <c r="D44" s="7">
+        <f>IF(OR(F8="",F8=0),"",D42/F8)</f>
+        <v/>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Expenses ÷ designers (Sedona 2026 had 16 paying designers)</t>
+        </is>
+      </c>
+    </row>
     <row r="45">
-      <c r="A45" s="10" t="inlineStr">
-        <is>
-          <t>YEAR 1 (2024), Cash vs. Donated</t>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Surplus From Prior Year</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n"/>
+      <c r="C45" s="5" t="n">
+        <v>5083</v>
+      </c>
+      <c r="D45" s="6" t="n"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>What was left in the bank from last year</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Cash Spent</t>
-        </is>
-      </c>
-      <c r="B46" s="11" t="n">
-        <v>2770</v>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Food, supplies, printing, VIP party</t>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>IN THE BANK AFTER</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="n"/>
+      <c r="C46" s="7">
+        <f>C45+C43</f>
+        <v/>
+      </c>
+      <c r="D46" s="7">
+        <f>D45+D43</f>
+        <v/>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Prior surplus + net. Sedona carried $4,723 into 2027</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Donated</t>
-        </is>
-      </c>
-      <c r="B47" s="11" t="n">
-        <v>6100</v>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Venue, sound / DJ, production help</t>
-        </is>
-      </c>
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>DONATED (IN-KIND) · not in the cash totals</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="n"/>
+      <c r="C47" s="4" t="n"/>
+      <c r="D47" s="4" t="n"/>
+      <c r="E47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Traded</t>
-        </is>
-      </c>
-      <c r="B48" s="11" t="n">
-        <v>997</v>
-      </c>
+          <t>Create-a-Thon Studio</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n"/>
+      <c r="C48" s="5" t="n">
+        <v>4800</v>
+      </c>
+      <c r="D48" s="6" t="n"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Venue hours swapped for services</t>
+          <t>Weekend studio space</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>Scholarship Courses &amp; Mentorship</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n"/>
+      <c r="C49" s="5" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D49" s="6" t="n"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Donated by the FABRIC Incubator</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Raffle Prizes</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n"/>
+      <c r="C50" s="5" t="n">
+        <v>6941</v>
+      </c>
+      <c r="D50" s="6" t="n"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>High-end items from local businesses</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Director / Producer Time</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n"/>
+      <c r="C51" s="5" t="n">
+        <v>4000</v>
+      </c>
+      <c r="D51" s="6" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n"/>
+      <c r="C52" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D52" s="6" t="n"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Two photographers</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Stage Manager</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n"/>
+      <c r="C53" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="D53" s="6" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n"/>
+      <c r="C54" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="D54" s="6" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>SAVED BY DONATIONS</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="n"/>
+      <c r="C55" s="7">
+        <f>SUM(C48:C54)</f>
+        <v/>
+      </c>
+      <c r="D55" s="7">
+        <f>SUM(D48:D54)</f>
+        <v/>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>What you didn't have to pay for</t>
+        </is>
+      </c>
+    </row>
+    <row r="56"/>
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>YEAR 1 (2024), Cash vs. Donated</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Cash Spent</t>
+        </is>
+      </c>
+      <c r="B58" s="11" t="n">
+        <v>2770</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Food, supplies, printing, VIP party</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Donated</t>
+        </is>
+      </c>
+      <c r="B59" s="11" t="n">
+        <v>6100</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Venue, sound / DJ, production help</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Traded</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="n">
+        <v>997</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Venue hours swapped for services</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>Value of the First Show</t>
         </is>
       </c>
-      <c r="B49" s="11" t="n">
+      <c r="B61" s="11" t="n">
         <v>10155</v>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>Before discounts and donations</t>
         </is>

</xml_diff>